<commit_message>
Add combination rows and bold-on-reference to output
- reference_amount.xlsx: add 'Includiert' column (col C) with semicolon-
  separated component section names for 4 new combination rows
  (Interventionen, Roe/CT ZNS und Skelett, Roe/CT Thorax -Organe Hals,
  Roe/CT/DL Abdomen Becken Retroperit)
- input_handler.py: add load_reference_data() returning amounts +
  combinations + ordered section list; load_reference_amounts() is now a
  backward-compatible wrapper
- output_handler.py: combination rows show component values separated by
  ';', dropped when any component is missing; rows with a reference amount
  are rendered bold; ISNUMBER guard added to CF formulas; output order
  follows reference file
- main.py: switch from load_reference_amounts to load_reference_data and
  pass reference_data to save_output

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference_amount.xlsx
+++ b/reference_amount.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\code\RadioBefundungszahlConverter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9336E4B-69E6-48B3-B3FC-925D4601348B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FABEF44-A4A0-4806-B3D1-238302BAA88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2567" yWindow="1527" windowWidth="19200" windowHeight="14473" xr2:uid="{7C7B4D74-82D9-468C-8437-FAE531A273BE}"/>
+    <workbookView xWindow="-80" yWindow="0" windowWidth="12960" windowHeight="15360" xr2:uid="{7C7B4D74-82D9-468C-8437-FAE531A273BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>DL Gefäße</t>
   </si>
@@ -138,6 +138,33 @@
   </si>
   <si>
     <t>Benötigt</t>
+  </si>
+  <si>
+    <t>Interventionen</t>
+  </si>
+  <si>
+    <t>Roe/CT ZNS und Skelett</t>
+  </si>
+  <si>
+    <t>Roe/CT Thorax, -Organe, Hals</t>
+  </si>
+  <si>
+    <t>Roe/CT/DL Abdomen, Becken, Retroperit</t>
+  </si>
+  <si>
+    <t>Rö Abdomen, Becken, Retroperit; CT Abdomen, Becken, Retroperit; DL Abdomen, Becken, Retroperit;</t>
+  </si>
+  <si>
+    <t>Rö Hals/Thorax; CT Hals/Thorax; CT Herz</t>
+  </si>
+  <si>
+    <t>CT ZNS; Rö ZNS; Rö Skelett; CT Skelett</t>
+  </si>
+  <si>
+    <t>Vask. Intervention; non-vask Intervention</t>
+  </si>
+  <si>
+    <t>Includiert</t>
   </si>
 </sst>
 </file>
@@ -536,210 +563,246 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15F3F82E-13BA-4DDA-AFB2-5C6EFC400F88}">
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="26.17578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.46875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="79.41015625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="C1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3">
+        <v>300</v>
+      </c>
+      <c r="C3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3">
+      <c r="B4">
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4">
+      <c r="B5">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A5" s="1" t="s">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A6" s="1" t="s">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A7" s="1" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B7">
+      <c r="B8">
         <v>3000</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A8" s="1" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A9" s="1" t="s">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A10" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A10" s="1" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A11" s="1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A11" s="1" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A12" s="1" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B12">
+      <c r="B13">
         <v>1500</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A13" s="1" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A14" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14">
+        <v>4000</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A15" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A14" s="1" t="s">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A16" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A15" s="1" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A17" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A16" s="1" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A18" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B16">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19">
         <v>4000</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A17" s="1" t="s">
+      <c r="C19" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A20" s="1" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A18" s="1" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A21" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B18">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A19" s="1" t="s">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A22" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A20" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A21" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B21">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A22" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.5">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="B23">
         <v>3000</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="C23" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A25" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A26" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A27" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A28" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A25" s="1" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A29" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B25">
-        <v>800</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A26" s="1" t="s">
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A30" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A27" s="1" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A31" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A28" s="1" t="s">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.5">
+      <c r="A32" s="1" t="s">
         <v>26</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A29" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A30" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A31" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.5">
-      <c r="A32" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A34" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A35" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A36" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A37" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B33">
+      <c r="B37">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed ref for gesamt
</commit_message>
<xml_diff>
--- a/reference_amount.xlsx
+++ b/reference_amount.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\code\RadioBefundungszahlConverter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FABEF44-A4A0-4806-B3D1-238302BAA88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1495EC8-42E4-42FF-9962-CDE800B1F550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="0" windowWidth="12960" windowHeight="15360" xr2:uid="{7C7B4D74-82D9-468C-8437-FAE531A273BE}"/>
+    <workbookView xWindow="3667" yWindow="2653" windowWidth="19200" windowHeight="13347" xr2:uid="{7C7B4D74-82D9-468C-8437-FAE531A273BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -53,9 +53,6 @@
     <t>Drainage</t>
   </si>
   <si>
-    <t>MRT</t>
-  </si>
-  <si>
     <t>MRT Prostata</t>
   </si>
   <si>
@@ -140,18 +137,6 @@
     <t>Benötigt</t>
   </si>
   <si>
-    <t>Interventionen</t>
-  </si>
-  <si>
-    <t>Roe/CT ZNS und Skelett</t>
-  </si>
-  <si>
-    <t>Roe/CT Thorax, -Organe, Hals</t>
-  </si>
-  <si>
-    <t>Roe/CT/DL Abdomen, Becken, Retroperit</t>
-  </si>
-  <si>
     <t>Rö Abdomen, Becken, Retroperit; CT Abdomen, Becken, Retroperit; DL Abdomen, Becken, Retroperit;</t>
   </si>
   <si>
@@ -165,6 +150,21 @@
   </si>
   <si>
     <t>Includiert</t>
+  </si>
+  <si>
+    <t>Interventionen gesamt</t>
+  </si>
+  <si>
+    <t>Roe/CT ZNS und Skelett gesamt</t>
+  </si>
+  <si>
+    <t>Roe/CT Thorax, -Organe, Hals gesamt</t>
+  </si>
+  <si>
+    <t>Roe/CT/DL Abdomen, Becken, Retroperit gesamt</t>
+  </si>
+  <si>
+    <t>MRT gesamt</t>
   </si>
 </sst>
 </file>
@@ -572,13 +572,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.5">
@@ -588,13 +588,13 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>300</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.5">
@@ -625,7 +625,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="B8">
         <v>3000</v>
@@ -633,27 +633,27 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13">
         <v>1500</v>
@@ -661,85 +661,85 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B14">
         <v>4000</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A17" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B19">
         <v>4000</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B23">
         <v>3000</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B26">
         <v>500</v>
@@ -747,7 +747,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B27">
         <v>800</v>
@@ -755,52 +755,52 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A29" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A30" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A31" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A32" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B37">
         <v>100</v>

</xml_diff>

<commit_message>
fixes gesamt in reference
</commit_message>
<xml_diff>
--- a/reference_amount.xlsx
+++ b/reference_amount.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sebas\code\RadioBefundungszahlConverter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FABEF44-A4A0-4806-B3D1-238302BAA88A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58711D8C-A9F2-4D44-BB08-2A2B198AA04F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="0" windowWidth="12960" windowHeight="15360" xr2:uid="{7C7B4D74-82D9-468C-8437-FAE531A273BE}"/>
+    <workbookView xWindow="1467" yWindow="1467" windowWidth="19200" windowHeight="13346" xr2:uid="{7C7B4D74-82D9-468C-8437-FAE531A273BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -53,9 +53,6 @@
     <t>Drainage</t>
   </si>
   <si>
-    <t>MRT</t>
-  </si>
-  <si>
     <t>MRT Prostata</t>
   </si>
   <si>
@@ -165,6 +162,9 @@
   </si>
   <si>
     <t>Includiert</t>
+  </si>
+  <si>
+    <t>MRT gesamt</t>
   </si>
 </sst>
 </file>
@@ -572,13 +572,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="C1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.5">
@@ -588,13 +588,13 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A3" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B3">
         <v>300</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.5">
@@ -625,7 +625,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A8" s="1" t="s">
-        <v>5</v>
+        <v>42</v>
       </c>
       <c r="B8">
         <v>3000</v>
@@ -633,27 +633,27 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A9" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A10" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A11" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A12" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A13" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13">
         <v>1500</v>
@@ -661,85 +661,85 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A14" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14">
         <v>4000</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A15" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A16" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A17" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A18" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A19" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B19">
         <v>4000</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A20" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A21" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A22" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A23" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B23">
         <v>3000</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A24" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A25" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A26" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B26">
         <v>500</v>
@@ -747,7 +747,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A27" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B27">
         <v>800</v>
@@ -755,52 +755,52 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A28" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A29" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A30" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A31" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.5">
       <c r="A32" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A33" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A34" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A35" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A36" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.5">
       <c r="A37" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B37">
         <v>100</v>

</xml_diff>